<commit_message>
feat: modernize frontend UI with immersive space theme, premium navigation, and optimized workflow
- Added NeuralNetworkBackground with twinkling stars, drifting nebulas, and mouse-reactive parallax\n- Implemented fixed glassmorphism header with scroll-spy, URL synchronization, and gradient progress bar\n- Relocated document processing pipeline and data correction table immediately after upload for contextual UX\n- Integrated official UPAY branding across the global navigation\n- Refactored contact section with real-time state management and frontend-only submission simulation\n- Ensured full theme-awareness for Light and Dark modes in all new components
</commit_message>
<xml_diff>
--- a/Scan-to-Excel/Backend/outputs/jte_output.xlsx
+++ b/Scan-to-Excel/Backend/outputs/jte_output.xlsx
@@ -505,14 +505,22 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>anushoce</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+          <t>Tanushree</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>7:45</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>1st</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">

</xml_diff>